<commit_message>
Folha «Resposta UPE» também na sincronização do mestre
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012uxwqH5ZwUWosxzcs9nhPb
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 16h33 UTC</t>
+          <t>26/10/2026, 16h36 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -3332,7 +3332,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 16h33 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 16h36 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
calibração 2026-10-26 18:41 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AN$5001</definedName>
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 16h36 UTC</t>
+          <t>26/10/2026, 18h41 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -3332,7 +3332,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 16h36 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 18h41 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-26 18:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 18h41 UTC</t>
+          <t>26/10/2026, 18h43 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2827,7 +2827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2867,73 +2867,121 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2946,7 +2994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3266,17 +3314,17 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Parecer CFP - Previsões macroeconómicas subjacentes à Proposta de Orçamento do Estado para 2027</t>
+          <t>Parecer ANMP - Associação Nacional de Municípios Portugueses</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=hgfi1mTNXDwia4mp6cO0KyoSVDQlWRwqRaWgQyiH77Oc%2bazA7FRl7v%2fzcSnnF3w3ERJrvARf27qxeRO2fv5BNI3jxRB8SLIn3hlgxVE2oSMoWGxWvfWJWRPoIcZuRU2QKxZ6HWsFP8o5gt6%2fdilusWIS3d3f2K1eaMYaZseldp14n24dxhnA015pYtWugitdrBBXKKQ1fTMPilXVSOloMYt6Jq0NDJ5pagMATvLNJNZi%2bG711rXGoy1CnhEADq5CRmYb%2fKpGkoeaApvCYRLBTLpdQBby1Qsne34MBGCLNYaNXJaIhQcT5jD0HaOkcjI1&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=tLjfmAPlmVlGyU3%2byXmB6PxP6K9YASTVFNZGHtjb1b2rArS8dcgJfLejoiyVM6mPl1aTKUin3DsGIvtNylyQTrCpl7EyJW%2bA3%2fUhFMhFLTLtAr0CMQEVG6%2fpsFcWU35S4IWdEVKlWzi3It%2f8HUfvQA81MFT6CkBaywQsyRUxUvW9Ws9NEaxDSrFujIxBSZwIu329hi3fFa0O7WjE6MGhFUr5x2%2f8mQ%2bVMEmfzHGtoCA8qBFeemtXnF7l5B%2bUVWywxEJgY1fTRSGczKzBfJS2pQuIYmc5VviiAC%2brs9EonmQHRpZfIevCqOpW%2b4MLGDgilCVLDYD8fJmk5BEUt64SNDsHNwiHYNqkEXXzcx6IQFgd2w%2baQc6%2fnpCEZyiuogIJ&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Registado no painel em 2026-10-26 04:39</t>
+          <t>Registado no painel em 2026-10-26 18:43</t>
         </is>
       </c>
     </row>
@@ -3288,15 +3336,59 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
+          <t>Relatório CFP - Análise da Proposta de Orçamento do Estado para 2027</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=jg0liXZh0D7ZDPOwFIxTR7RmQRG6jfgbSD1YLR86ni7XOo%2fGHAe10dYNOKlomIDVod8axty1H%2brKtWtOSyL%2bEqsQyHsBcDWFk2WSYlnw%2fDHjzxXPCg9xvNXqp%2fieQgpzrNca6ZjESC2MqBXgFb9OmZlgujo5RhXK1WTGEHsnD%2beOlQQ7K23LOxnA9iGH3WnQ1TWNV05cFrTE6HSSWMj8S2xKfp0%2bAe8tI3bsqla1XR8l9wmq7%2fLDz9GCO4T2YXNYFUWfaEiSxDsgIwcJ%2fxe6UfdaiP7%2fgHwCWbvD1DclOmjsalowXN4MhguYV%2buR3niMOpmyB3KNVXkNVK%2fdoLZgV36IOPvIypzLcYsG%2bQvOyizqOwrYhQf1n1dtT3d5oaah&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Registado no painel em 2026-10-26 18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Parecer CFP - Previsões macroeconómicas subjacentes à Proposta de Orçamento do Estado para 2027</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=wc5A5hly7AavluyfljWjL4C5BRBMB9iGDv5qX606jn8oZJx1XeJl5Lyfwxbby1zM3PUh3feNHF4HxhdGSjRUcFKutVANdS41VfOsSp9HVFOBEozIH361AlnBhNSONHGVHVBpv9hf2wsQrYtEqryluvsr2oDKvTgp%2br%2b0Lhwsm1nZ4SuRnFdwxMnkJ4w9CIpBSbYtd9QMyiNmEe7oc9OZIXBEt%2f78EDzdIxu3QoOrRJkYXxU6%2bhhsxP6qiMJrUGCDADUVDNUCTLNAjVM%2f62%2f8wp6N4LEYTmL9MZ3u6M%2fJpYjfs62VLbTM6DoIuFYAGsR4A3z%2bE33YUex9fTD7ARoL2A%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Registado no painel em 2026-10-26 04:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
           <t>Relatório UTAO - Apreciação preliminar da Proposta de Orçamento do Estado para 2027</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=NzSH7u9fWS1pIol46TtMSjZPmPGhdgb8G6JQjh813HJZf%2bm2n5HU02v1OeuqwwJ7r%2bJtqRmpbssXFvz3uuZGdffLImxqTpEQZju%2f4I%2foucAApKAx%2b6BJ4SLx6llkOqq9uno%2fnUr%2bvGM1yU0s3ypCF3s5x5o0dCewIEjJ55kRTGs%2fNoJTGsNWnsIxMzuOdeV5E66qewYOyhCQuOl4MpYCW6fWDHKX9Ds2XG4gLUZRA0%2b33iawXVVc0cTHPiWpMnkTsIY%2bZ8FGbtEC1cAd%2bo9m5%2bZbzBO3DnxAL2ivFpT%2fpos225ozsJ2XKHuWIg2xKtK3HbdTIUsjYggaVErr7i%2fRYQ%3d%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=Y4RKE59ymJ2%2bcfR2U%2fv3ZFULw8umGJcbHe5gcCliOvpfpuFJ2DosjJWqbVrYGQSxf6My%2bRhIL85SorxHqJ%2bj2TRSzOD%2fQ6z3md5oPHWJKsag%2fI5EhOqVK1imbdOa70sLaKbLN%2bBTXYApROtkdvLoc1ohil9lRC8WdUGfGnJKLBrqiIEYJnw%2bnkDHYVGdb13vsr6zQMB2DaNMAZI3bCuLFbGJp8g4N7cfdaHvHXCunuAcI705LTRbF03ruOpHVkns1u0jG6MkiwXErNQkvPNyYWSYNXUPuRLVB0Z39NWNtfaCpWaEu6FDRWyNouvmyU4A909UmX3%2fkvmgQO1VTFPuNB7FcBcsNx93Q03z0wyKTxY%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Registado no painel em 2026-10-26 04:19</t>
         </is>
@@ -3332,7 +3424,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 18h41 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 18h43 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
calibração 2026-10-26 18:44 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 18h43 UTC</t>
+          <t>26/10/2026, 18h44 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -3424,7 +3424,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 18h43 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 18h44 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-26 18:46 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 18h44 UTC</t>
+          <t>26/10/2026, 18h46 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2827,7 +2827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2867,121 +2867,169 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3424,7 +3472,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 18h44 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 18h46 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-26 18:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 18h46 UTC</t>
+          <t>26/10/2026, 18h48 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2827,7 +2827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2867,7 +2867,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2892,7 +2892,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2915,121 +2915,169 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E8" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3472,7 +3520,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 18h46 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 18h48 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
Painel e Excel só com variáveis dos dados abertos da AR: retirada a área governativa (fase posterior, com validação humana); posição dos grupos parlamentares por tema da AR
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012uxwqH5ZwUWosxzcs9nhPb
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AN$5001</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AJ$5001</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Medidas Anunciadas'!$A$1:$M$5001</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN2"/>
+  <dimension ref="A1:AJ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -495,22 +495,18 @@
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="40" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="26" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="22" customWidth="1" min="30" max="30"/>
-    <col width="24" customWidth="1" min="31" max="31"/>
-    <col width="10" customWidth="1" min="32" max="32"/>
-    <col width="7" customWidth="1" min="33" max="33"/>
-    <col width="9" customWidth="1" min="34" max="34"/>
-    <col width="9" customWidth="1" min="35" max="35"/>
-    <col width="40" customWidth="1" min="36" max="36"/>
-    <col width="40" customWidth="1" min="37" max="37"/>
-    <col width="17" customWidth="1" min="38" max="38"/>
-    <col width="17" customWidth="1" min="39" max="39"/>
-    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="7" customWidth="1" min="29" max="29"/>
+    <col width="9" customWidth="1" min="30" max="30"/>
+    <col width="9" customWidth="1" min="31" max="31"/>
+    <col width="40" customWidth="1" min="32" max="32"/>
+    <col width="40" customWidth="1" min="33" max="33"/>
+    <col width="17" customWidth="1" min="34" max="34"/>
+    <col width="17" customWidth="1" min="35" max="35"/>
+    <col width="17" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -636,80 +632,60 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Área Governativa (sugestão SGGov)</t>
+          <t>Incide</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Método da sugestão</t>
+          <t>Tipo (AR)</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Confiança</t>
+          <t>Estado (AR)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Tipo de PA (sugestão)</t>
+          <t>Avocação a Plenário</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Incide</t>
+          <t>Parte</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Tipo (AR)</t>
+          <t>N.º de votações</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Estado (AR)</t>
+          <t>ID AR</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Avocação a Plenário</t>
+          <t>Ligação AR</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Parte</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>N.º de votações</t>
+          <t>Primeira captura</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>ID AR</t>
+          <t>Última captura</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>Ligação AR</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>Primeira captura</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>Última captura</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Ausente da fonte</t>
         </is>
@@ -749,16 +725,12 @@
       <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
       <c r="AG2" s="2" t="n"/>
-      <c r="AH2" s="2" t="n"/>
-      <c r="AI2" s="2" t="n"/>
+      <c r="AH2" s="3" t="n"/>
+      <c r="AI2" s="3" t="n"/>
       <c r="AJ2" s="2" t="n"/>
-      <c r="AK2" s="2" t="n"/>
-      <c r="AL2" s="3" t="n"/>
-      <c r="AM2" s="3" t="n"/>
-      <c r="AN2" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN5001"/>
+  <autoFilter ref="A1:AJ5001"/>
   <dataValidations count="8">
     <dataValidation sqref="D2:D5001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$A$2:$A$4</formula1>
@@ -893,7 +865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -920,7 +892,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 18h48 UTC</t>
+          <t>26/10/2026, 21h59 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -1500,386 +1472,6 @@
       <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="n"/>
       <c r="D40" s="2" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Por área governativa (sugestão SGGov, coluna Y; substituir pela coluna J quando validada pela DACDP)</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Área governativa</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>N.º PA</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Aprovadas</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Rejeitadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Presidência</t>
-        </is>
-      </c>
-      <c r="B44" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A44)</f>
-        <v/>
-      </c>
-      <c r="C44" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A44,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D44" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A44,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Estado e Finanças</t>
-        </is>
-      </c>
-      <c r="B45" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A45)</f>
-        <v/>
-      </c>
-      <c r="C45" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A45,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D45" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A45,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Estado e Negócios Estrangeiros</t>
-        </is>
-      </c>
-      <c r="B46" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A46)</f>
-        <v/>
-      </c>
-      <c r="C46" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A46,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D46" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A46,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Adjunto e Reforma do Estado</t>
-        </is>
-      </c>
-      <c r="B47" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A47)</f>
-        <v/>
-      </c>
-      <c r="C47" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A47,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D47" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A47,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Assuntos Parlamentares</t>
-        </is>
-      </c>
-      <c r="B48" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A48)</f>
-        <v/>
-      </c>
-      <c r="C48" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A48,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D48" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A48,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Defesa Nacional</t>
-        </is>
-      </c>
-      <c r="B49" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A49)</f>
-        <v/>
-      </c>
-      <c r="C49" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A49,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D49" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A49,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Administração Interna</t>
-        </is>
-      </c>
-      <c r="B50" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A50)</f>
-        <v/>
-      </c>
-      <c r="C50" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A50,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D50" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A50,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Justiça</t>
-        </is>
-      </c>
-      <c r="B51" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A51)</f>
-        <v/>
-      </c>
-      <c r="C51" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A51,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D51" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A51,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Economia e Coesão Territorial</t>
-        </is>
-      </c>
-      <c r="B52" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A52)</f>
-        <v/>
-      </c>
-      <c r="C52" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A52,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D52" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A52,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Educação, Ciência e Inovação</t>
-        </is>
-      </c>
-      <c r="B53" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A53)</f>
-        <v/>
-      </c>
-      <c r="C53" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A53,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D53" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A53,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Saúde</t>
-        </is>
-      </c>
-      <c r="B54" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A54)</f>
-        <v/>
-      </c>
-      <c r="C54" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A54,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D54" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A54,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Infraestruturas e Habitação</t>
-        </is>
-      </c>
-      <c r="B55" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A55)</f>
-        <v/>
-      </c>
-      <c r="C55" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A55,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D55" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A55,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Trabalho, Solidariedade e Segurança Social</t>
-        </is>
-      </c>
-      <c r="B56" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A56)</f>
-        <v/>
-      </c>
-      <c r="C56" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A56,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D56" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A56,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Ambiente e Energia</t>
-        </is>
-      </c>
-      <c r="B57" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A57)</f>
-        <v/>
-      </c>
-      <c r="C57" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A57,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D57" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A57,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Agricultura e Mar</t>
-        </is>
-      </c>
-      <c r="B58" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A58)</f>
-        <v/>
-      </c>
-      <c r="C58" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A58,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D58" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A58,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Cultura, Juventude e Desporto</t>
-        </is>
-      </c>
-      <c r="B59" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A59)</f>
-        <v/>
-      </c>
-      <c r="C59" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A59,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D59" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A59,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="B60" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A60)</f>
-        <v/>
-      </c>
-      <c r="C60" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A60,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D60" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A60,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>por classificar</t>
-        </is>
-      </c>
-      <c r="B61" s="2">
-        <f>COUNTIF('Propostas de Alteração'!$Y$2:$Y$5001,A61)</f>
-        <v/>
-      </c>
-      <c r="C61" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A61,'Propostas de Alteração'!$T$2:$T$5001,"Aprovada")</f>
-        <v/>
-      </c>
-      <c r="D61" s="2">
-        <f>COUNTIFS('Propostas de Alteração'!$Y$2:$Y$5001,A61,'Propostas de Alteração'!$T$2:$T$5001,"Rejeitada")</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2718,7 +2310,7 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>As colunas B, C, E, F, G, L, S, T, U e V e as ligações em W são preenchidas a partir da Assembleia da República em cada captura automática. As colunas X em diante são informação adicional da UPE: tema atribuído pela AR, sugestão de área governativa (classificação SGGov, com método e confiança), sugestão de tipo, avocação, identificadores e ligações. As restantes colunas do modelo (D, H a K, M a R e o texto de W) são da DACDP e nunca são alteradas pela sincronização.</t>
+          <t>As colunas B, C, E, F, G, L, S, T, U e V e as ligações em W são preenchidas a partir dos dados abertos da Assembleia da República em cada captura automática. As colunas X em diante são informação adicional publicada pela AR: tema, incidência, natureza e estado da PA, avocação, identificadores e ligações. As restantes colunas do modelo (D, H a K, M a R e o texto de W) são da DACDP e nunca são alteradas pela sincronização.</t>
         </is>
       </c>
       <c r="B30" s="8" t="n"/>
@@ -3520,7 +3112,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 18h48 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 21h59 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>
@@ -3621,12 +3213,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Limitação</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>A AR não liga uma PA à que ela substitui. A UPE assinala candidatas (mesmo proponente e artigo, uma retirada e outra posterior) em Observações.</t>
+          <t>A AR não publica a ligação entre uma PA e a que ela substitui. A coluna recebe «Retirada» quando a AR publica esse estado e «Original» nos restantes casos.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -3701,17 +3293,17 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Limitação</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Sugestão por regra nos casos claros (mapas de receita e despesa, autorizações legislativas, alterações a códigos e leis avulsas), na coluna «Tipo de PA (sugestão)».</t>
+          <t>Sem fonte na AR (a AR publica a natureza da PA: aditamento, substituição, eliminação, na coluna «Tipo (AR)»).</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Leitura humana nos restantes casos.</t>
+          <t>Classificação da DACDP. Fase posterior: sugestão automática a validar.</t>
         </is>
       </c>
     </row>
@@ -3741,17 +3333,17 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Desenvolvimento (fase posterior)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Sugestão SGGov na coluna «Área Governativa (sugestão SGGov)»: tabela artigo → área (feita uma vez por ano), programa orçamental nos mapas e palavras-chave; método e confiança indicados.</t>
+          <t>Sem fonte na AR. O tema atribuído pela AR (coluna «Tema AR», a comissão parlamentar competente) é a aproximação disponível. A classificação por área governativa será feita numa fase posterior, com validação humana.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Validação pela DACDP. A classificação validada volta ao painel, assinalada como classificação DACDP.</t>
+          <t>Nesta fase, o painel e o Excel só usam variáveis dos dados abertos da AR.</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3355,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Desenvolvimento (fase posterior)</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3857,19 +3449,15 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Limitação</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Sugestão por semelhança entre o título da PA e as medidas da folha «Medidas Anunciadas».</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>A ligação é juízo da DACDP.</t>
-        </is>
-      </c>
+          <t>Sem fonte na AR. Ligação à folha «Medidas Anunciadas» pelo n.º da PA, a cargo da DACDP.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -3897,19 +3485,15 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Limitação</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Sugestão «S» quando a PA altera legislação avulsa.</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Juízo da DACDP nos restantes casos.</t>
-        </is>
-      </c>
+          <t>Juízo da DACDP.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">

</xml_diff>

<commit_message>
captura 2026-10-26 22:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AJ$5001</definedName>
@@ -892,7 +892,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 21h59 UTC</t>
+          <t>26/10/2026, 22h01 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2419,7 +2419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2459,7 +2459,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2484,7 +2484,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2532,7 +2532,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2555,121 +2555,169 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3007,7 +3055,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=tLjfmAPlmVlGyU3%2byXmB6PxP6K9YASTVFNZGHtjb1b2rArS8dcgJfLejoiyVM6mPl1aTKUin3DsGIvtNylyQTrCpl7EyJW%2bA3%2fUhFMhFLTLtAr0CMQEVG6%2fpsFcWU35S4IWdEVKlWzi3It%2f8HUfvQA81MFT6CkBaywQsyRUxUvW9Ws9NEaxDSrFujIxBSZwIu329hi3fFa0O7WjE6MGhFUr5x2%2f8mQ%2bVMEmfzHGtoCA8qBFeemtXnF7l5B%2bUVWywxEJgY1fTRSGczKzBfJS2pQuIYmc5VviiAC%2brs9EonmQHRpZfIevCqOpW%2b4MLGDgilCVLDYD8fJmk5BEUt64SNDsHNwiHYNqkEXXzcx6IQFgd2w%2baQc6%2fnpCEZyiuogIJ&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=%2fpNClpGGPpVnhbwFVXgp4qw3lFxiUpY5I8YSpeDVGH2Ez9MewVxhJZgmbME%2fa6%2bTMjV1mONPHi9qMLwrLk3vT83H5KkhIuSYQfR80BVPktegQ7Gl%2fwLhJpBRS2u1cG5OhrLVdG2YC%2bJsQxSRbcR72ynl4Szw0Kx5iDcONLD%2bGFkQ9jwIhmEnb9oj7mBISGyCnFAW%2boWpZ6JJhPzu0o0Y5y4ZJpvJ2OuBmMNL%2feYLRFY1wbMgbEZlgt35l6hrfQiWUu1j5GiKwdCYdJ9xj%2bC1ffYEAfCP0FxQup9C8cKn6PXPJ%2fcBQEZ6o%2b1Iaq9a4krvJL2CejZIuZgnT0UudK%2bZZNY47LDueTbwPwP4xVZ8KQ0J%2bQUo0RpWw0P8BT%2f3DmTE&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3029,7 +3077,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=jg0liXZh0D7ZDPOwFIxTR7RmQRG6jfgbSD1YLR86ni7XOo%2fGHAe10dYNOKlomIDVod8axty1H%2brKtWtOSyL%2bEqsQyHsBcDWFk2WSYlnw%2fDHjzxXPCg9xvNXqp%2fieQgpzrNca6ZjESC2MqBXgFb9OmZlgujo5RhXK1WTGEHsnD%2beOlQQ7K23LOxnA9iGH3WnQ1TWNV05cFrTE6HSSWMj8S2xKfp0%2bAe8tI3bsqla1XR8l9wmq7%2fLDz9GCO4T2YXNYFUWfaEiSxDsgIwcJ%2fxe6UfdaiP7%2fgHwCWbvD1DclOmjsalowXN4MhguYV%2buR3niMOpmyB3KNVXkNVK%2fdoLZgV36IOPvIypzLcYsG%2bQvOyizqOwrYhQf1n1dtT3d5oaah&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=ssTiMSuZoJCViNd1vgR6NWHID3MGPk8ccDEG8T7aT7Knp0%2bD6ahQu3bm%2fXCAwHHP1m%2fLGYhARXLAI44s4yAdjFofVkflLmuhod%2fChfVb6xrtp%2fX8E1KGoSx5kEmueS0kHHfbLIBo7vFuQZD061hacolSP4UzHNsVtTsIZ%2bxqZa3NOtGWvlskniFr%2bqYioKXSCT2nZU7PsqRlrbtSWquK1%2fm5%2fSMMlkbw6t70dHBENjjqgCf6FVWAmkJfMfsWN06%2fwg1KFC9TCcBMPFlHWrC8bdy%2fMiGGFBX6YK09SuoPXLT6ExiRtSPYZpCeIB%2fZvqBhyiydH19tPstVSEMM8IKWo8Z0vwmgtxjhCAIi2zuiTBc%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -3051,7 +3099,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=wc5A5hly7AavluyfljWjL4C5BRBMB9iGDv5qX606jn8oZJx1XeJl5Lyfwxbby1zM3PUh3feNHF4HxhdGSjRUcFKutVANdS41VfOsSp9HVFOBEozIH361AlnBhNSONHGVHVBpv9hf2wsQrYtEqryluvsr2oDKvTgp%2br%2b0Lhwsm1nZ4SuRnFdwxMnkJ4w9CIpBSbYtd9QMyiNmEe7oc9OZIXBEt%2f78EDzdIxu3QoOrRJkYXxU6%2bhhsxP6qiMJrUGCDADUVDNUCTLNAjVM%2f62%2f8wp6N4LEYTmL9MZ3u6M%2fJpYjfs62VLbTM6DoIuFYAGsR4A3z%2bE33YUex9fTD7ARoL2A%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=fGXILUp6%2byvRm6Ifi40G9mUnq0dA55wCevtvBwtCMyx7gYlSzGO8j%2fN3obKpbXemnK2eBIpyO4lLCcO0rlA3hYaXLLW89UATI99Thh1jYaUEYYlK1%2bNIKAWZ%2fJ99%2feBnI0rhRr8020%2b4vwYeICKMx5GMs30mmbeZXKshd5E0izl2YNczd%2faDXHNQJMNQbuuXBqLXFSWZi9G2kkSltz%2bmJWmnu1W%2bRa9edq2a%2fbH1zlSEIktrSJBGGpPZVwHsz%2fOVEWMjrHQaVakyu15C1fzzMPR3BbC68LoFVnUZL%2f8xJJAWjadnHxGj7cG%2bRe42Ve4kxyzym7XK0H4drrQWGgjbZg%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3073,7 +3121,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=Y4RKE59ymJ2%2bcfR2U%2fv3ZFULw8umGJcbHe5gcCliOvpfpuFJ2DosjJWqbVrYGQSxf6My%2bRhIL85SorxHqJ%2bj2TRSzOD%2fQ6z3md5oPHWJKsag%2fI5EhOqVK1imbdOa70sLaKbLN%2bBTXYApROtkdvLoc1ohil9lRC8WdUGfGnJKLBrqiIEYJnw%2bnkDHYVGdb13vsr6zQMB2DaNMAZI3bCuLFbGJp8g4N7cfdaHvHXCunuAcI705LTRbF03ruOpHVkns1u0jG6MkiwXErNQkvPNyYWSYNXUPuRLVB0Z39NWNtfaCpWaEu6FDRWyNouvmyU4A909UmX3%2fkvmgQO1VTFPuNB7FcBcsNx93Q03z0wyKTxY%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=vIA7IukVsFL8hpTbQ2OM5whL1GkackwVcIcDmm6o5EWFIW5LSWyS7tEnH6b%2fJjhuVT59PCePI40rPmpxklo96oV%2bcFVfM1h7cjJ55RpcCH2VqQLpLcEaM%2fUy0Mj9%2fo12tFQ1m4960rvwIaJcQXSkd3ZraSglMqfe7kHTQr2pZhSKT%2bNuS7KluOGtL%2boO4e6PLS7%2bW8VPSJjXFJ0I3d5qUILDdrSN5BoFcS0CANXbN0d%2bbo3RoTfhTPj2ua4G3ns5RxjNRajHEgGNqtQzvpoudaIi2NIyOZD4wtCBGEpp9XkVp3wsZB9X8ge3HV7pA3eoLNEBhqAXARLQ%2btqXl5WHGJ1YmEzmS5hBbhTf2kGROOo%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3112,7 +3160,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 21h59 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h01 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
calibração 2026-10-26 22:03 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -892,7 +892,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h01 UTC</t>
+          <t>26/10/2026, 22h03 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -3160,7 +3160,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h01 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h03 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
Painel: separador «Por tema» (tema atribuído pela AR), ligações aos dados abertos no cabeçalho e nas fontes, ícone claro/escuro corrigido; sem referências à área governativa
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012uxwqH5ZwUWosxzcs9nhPb
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AJ$5001</definedName>
@@ -731,7 +731,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AJ5001"/>
-  <dataValidations count="8">
+  <dataValidations count="7">
     <dataValidation sqref="D2:D5001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$A$2:$A$4</formula1>
     </dataValidation>
@@ -752,9 +752,6 @@
     </dataValidation>
     <dataValidation sqref="T2:T5001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$G$2:$G$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J5001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Listas!$H$2:$H$18</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -892,7 +889,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h03 UTC</t>
+          <t>26/10/2026, 22h05 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -1484,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1494,7 +1491,6 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1533,11 +1529,6 @@
           <t>Resultado</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>Área Governativa</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1575,11 +1566,6 @@
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Presidência</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1617,11 +1603,6 @@
           <t>Rejeitada</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Estado e Finanças</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1654,11 +1635,6 @@
           <t>Prejudicada</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Estado e Negócios Estrangeiros</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
@@ -1681,11 +1657,6 @@
           <t>Retirada</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Adjunto e Reforma do Estado</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
@@ -1708,11 +1679,6 @@
           <t>Aprovada parcialmente</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Assuntos Parlamentares</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
@@ -1725,11 +1691,6 @@
           <t>Votada</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Defesa Nacional</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
@@ -1742,11 +1703,6 @@
           <t>Avocada a Plenário</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Administração Interna</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
@@ -1754,11 +1710,6 @@
           <t>BE</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Justiça</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
@@ -1766,11 +1717,6 @@
           <t>PAN</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Economia e Coesão Territorial</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
@@ -1778,11 +1724,6 @@
           <t>JPP</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Educação, Ciência e Inovação</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
@@ -1790,56 +1731,11 @@
           <t>Deputado único/não inscrito</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Saúde</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Vários</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Infraestruturas e Habitação</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Trabalho, Solidariedade e Segurança Social</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Ambiente e Energia</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Agricultura e Mar</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Cultura, Juventude e Desporto</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Transversal</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3056,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h03 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h05 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>
@@ -3351,7 +3247,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Classificação da DACDP. Fase posterior: sugestão automática a validar.</t>
+          <t>Classificação da DACDP.</t>
         </is>
       </c>
     </row>
@@ -3381,17 +3277,17 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento (fase posterior)</t>
+          <t>Limitação</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Sem fonte na AR. O tema atribuído pela AR (coluna «Tema AR», a comissão parlamentar competente) é a aproximação disponível. A classificação por área governativa será feita numa fase posterior, com validação humana.</t>
+          <t>Sem fonte na AR. O tema atribuído pela AR (coluna «Tema AR»; em 2026, a comissão parlamentar competente) é a aproximação disponível.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Nesta fase, o painel e o Excel só usam variáveis dos dados abertos da AR.</t>
+          <t>Classificação da DACDP.</t>
         </is>
       </c>
     </row>
@@ -3403,15 +3299,19 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvimento (fase posterior)</t>
+          <t>Limitação</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Decorre da área governativa.</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr"/>
+          <t>Sem fonte na AR.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Classificação da DACDP.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">

</xml_diff>

<commit_message>
captura 2026-10-26 22:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AJ$5001</definedName>
@@ -889,7 +889,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h05 UTC</t>
+          <t>26/10/2026, 22h07 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2315,7 +2315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2355,7 +2355,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2380,7 +2380,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2403,7 +2403,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2451,7 +2451,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2476,7 +2476,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2499,121 +2499,169 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E12" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2951,7 +2999,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=%2fpNClpGGPpVnhbwFVXgp4qw3lFxiUpY5I8YSpeDVGH2Ez9MewVxhJZgmbME%2fa6%2bTMjV1mONPHi9qMLwrLk3vT83H5KkhIuSYQfR80BVPktegQ7Gl%2fwLhJpBRS2u1cG5OhrLVdG2YC%2bJsQxSRbcR72ynl4Szw0Kx5iDcONLD%2bGFkQ9jwIhmEnb9oj7mBISGyCnFAW%2boWpZ6JJhPzu0o0Y5y4ZJpvJ2OuBmMNL%2feYLRFY1wbMgbEZlgt35l6hrfQiWUu1j5GiKwdCYdJ9xj%2bC1ffYEAfCP0FxQup9C8cKn6PXPJ%2fcBQEZ6o%2b1Iaq9a4krvJL2CejZIuZgnT0UudK%2bZZNY47LDueTbwPwP4xVZ8KQ0J%2bQUo0RpWw0P8BT%2f3DmTE&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=OsCemGn18KHljJghQ1ajbT%2fWEjfWtVhYUV7kRe%2fuHXhoN3nBlFtEOKbVu6QDIijjtsN4R56fyr1%2baHaxmvmZpOEUCWUfOUfj3wrrcEwZ7N0EVKamFEyyE1w79r%2bkbcYOysKTZQ%2frSXfq8yeBOh6uz%2bSSo7dNrYki3milkOdQK4%2fPYhVDAHRIYYyOrz9AfNYHC6%2bLY7wFcjRBgKXEr2gBz6WFsM9%2f%2bww2K4Y5MtDusKVrhlNwfEP%2bBxwqxK3ENqiwcJoPZY%2bbUiARod2nAS1emsn6ZnlYZFQfTpmOOV%2fbDqZGELEKpDw3plGCXSPbL7OVXVY4RzOCwW0D3v8CPMBJ6J1Zybv%2bENyPWZ7DPH8OTuQ%3d&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -2973,7 +3021,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=ssTiMSuZoJCViNd1vgR6NWHID3MGPk8ccDEG8T7aT7Knp0%2bD6ahQu3bm%2fXCAwHHP1m%2fLGYhARXLAI44s4yAdjFofVkflLmuhod%2fChfVb6xrtp%2fX8E1KGoSx5kEmueS0kHHfbLIBo7vFuQZD061hacolSP4UzHNsVtTsIZ%2bxqZa3NOtGWvlskniFr%2bqYioKXSCT2nZU7PsqRlrbtSWquK1%2fm5%2fSMMlkbw6t70dHBENjjqgCf6FVWAmkJfMfsWN06%2fwg1KFC9TCcBMPFlHWrC8bdy%2fMiGGFBX6YK09SuoPXLT6ExiRtSPYZpCeIB%2fZvqBhyiydH19tPstVSEMM8IKWo8Z0vwmgtxjhCAIi2zuiTBc%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=pYwL3M4UXS4UTKShXKrBwWhp6ojHm69gObwqFN1l2E%2bxg2kG%2fhptXWmW2pG0nq46Z59GR5Hv4XPds%2bZNQrAz4A2DsnQmjHZ7PCKqj18SSwmD98VOnInmTVCdi3ITI6c4SpPPqKeXEmPQpLXOseTAjZizKS46mKyrfyKCMffvgYdbTSGC%2fbxtvJLWsGKsUDEiy0HElY9pnszJB5Bjl10iuYYp2j%2fFkyqILEqiR6F9Qx0MhMQNVRBAGgk0atcvWXLKrHuW7BV8WWt%2bQ9OGXY3m5RhVZXQ0lAc8%2bKQzNNQF1Jw271ya0A%2fQ5zo978ZcQ9MItZ6V%2fdGbJOsCxE%2filt86HDnv0Mwioj9hwHnFYJNfUgI%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -2995,7 +3043,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=fGXILUp6%2byvRm6Ifi40G9mUnq0dA55wCevtvBwtCMyx7gYlSzGO8j%2fN3obKpbXemnK2eBIpyO4lLCcO0rlA3hYaXLLW89UATI99Thh1jYaUEYYlK1%2bNIKAWZ%2fJ99%2feBnI0rhRr8020%2b4vwYeICKMx5GMs30mmbeZXKshd5E0izl2YNczd%2faDXHNQJMNQbuuXBqLXFSWZi9G2kkSltz%2bmJWmnu1W%2bRa9edq2a%2fbH1zlSEIktrSJBGGpPZVwHsz%2fOVEWMjrHQaVakyu15C1fzzMPR3BbC68LoFVnUZL%2f8xJJAWjadnHxGj7cG%2bRe42Ve4kxyzym7XK0H4drrQWGgjbZg%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=Prp2%2b5ePDHjXkp5VUsQPct9bJa2RQHLO%2fyYIuha7TLAa8p6hUj1fY7Fe%2fZGk9wbXwEZmw1S14NL4ZNI8VLtcauMrxEYr0JWlnK6gPBDY3p4njYtKa%2fqnpDDAMqJEZq19UxZT6D1kt8yXuKOVU7m%2bSauySQ7xuQrqKKi11B4UGS6E%2bqkaNhmxoIqJD8U%2bCBEMrKZtj%2bAZTOvjMRpQ75atN0haT3lT67EnV7grLUcEz4%2f%2b0YUjA1h11II2KmNjheJuizQ1x3Z0c2mtgzKFJ%2fukV3duaJOIlcVz5WQbKzQvp%2fr3N7GFi3WPm15oMGmVQuTL4Iu8uiZpGwWXooc9EtWsty1Z2nzbXVJuYAv66%2f77LXc%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3017,7 +3065,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=vIA7IukVsFL8hpTbQ2OM5whL1GkackwVcIcDmm6o5EWFIW5LSWyS7tEnH6b%2fJjhuVT59PCePI40rPmpxklo96oV%2bcFVfM1h7cjJ55RpcCH2VqQLpLcEaM%2fUy0Mj9%2fo12tFQ1m4960rvwIaJcQXSkd3ZraSglMqfe7kHTQr2pZhSKT%2bNuS7KluOGtL%2boO4e6PLS7%2bW8VPSJjXFJ0I3d5qUILDdrSN5BoFcS0CANXbN0d%2bbo3RoTfhTPj2ua4G3ns5RxjNRajHEgGNqtQzvpoudaIi2NIyOZD4wtCBGEpp9XkVp3wsZB9X8ge3HV7pA3eoLNEBhqAXARLQ%2btqXl5WHGJ1YmEzmS5hBbhTf2kGROOo%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=8VcRHu%2fGqpM4lRNrVpi9AeQ4K1Q9SnoLZ8akeOecC5sq918XRI4NEQkNDDgMmi1KupFpJ96lD21jWApIA118S9VBF4z6dlOVujEnpf2Ne3BCAIJtHbrVLchFqP%2bRWhnF%2bkAsDUaroQYYKdn0aqeiW9rRlDaUkJHWjgDNyZDu8nPITgU%2bKoG9jKrSGdrE68ioXc5QFZIbFjVs38td%2feKpMKELaoSWqIFqRqBqqyhvrXSzL%2b96AAETfgV8UkPVEmg5Wz06eSb6bsqQiuaPcs%2bOuyq9lNF1qFsUkh6H6%2bI9sJO9%2bnP%2fji0rTJramuKoYFbqHbBa6IH0aHyGMfq9JEcY8Q%3d%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3056,7 +3104,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h05 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h07 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
Painel redesenhado: separadores fixos, modo claro/escuro explícito, hero com distribuição de estados, barras empilhadas por resultado, gráficos de entradas por dia e por hora, cores dos partidos, ligações profundas (#oe2026/temas), impressão A4 horizontal com cores; contagens pela convenção da AR; novos campos da AR (epígrafe, diplomas, requerimentos, parecer RA, ministério); verificações automáticas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012uxwqH5ZwUWosxzcs9nhPb
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AJ$5001</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AO$5001</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Medidas Anunciadas'!$A$1:$M$5001</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ2"/>
+  <dimension ref="A1:AO2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -495,18 +495,23 @@
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="40" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="10" customWidth="1" min="28" max="28"/>
-    <col width="7" customWidth="1" min="29" max="29"/>
-    <col width="9" customWidth="1" min="30" max="30"/>
-    <col width="9" customWidth="1" min="31" max="31"/>
-    <col width="40" customWidth="1" min="32" max="32"/>
-    <col width="40" customWidth="1" min="33" max="33"/>
-    <col width="17" customWidth="1" min="34" max="34"/>
-    <col width="17" customWidth="1" min="35" max="35"/>
-    <col width="17" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="30" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="7" customWidth="1" min="34" max="34"/>
+    <col width="9" customWidth="1" min="35" max="35"/>
+    <col width="9" customWidth="1" min="36" max="36"/>
+    <col width="40" customWidth="1" min="37" max="37"/>
+    <col width="40" customWidth="1" min="38" max="38"/>
+    <col width="17" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="17" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -632,60 +637,85 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>Epígrafe do artigo (AR)</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Diplomas alterados (AR)</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>Incide</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Tipo (AR)</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Estado (AR)</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Avocação a Plenário</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Requerimentos (AR)</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Parecer Regiões Autónomas (AR)</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Ministério (AR)</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Parte</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>N.º de votações</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>ID AR</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Ligação AR</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Primeira captura</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Última captura</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Ausente da fonte</t>
         </is>
@@ -725,12 +755,17 @@
       <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
       <c r="AG2" s="2" t="n"/>
-      <c r="AH2" s="3" t="n"/>
-      <c r="AI2" s="3" t="n"/>
+      <c r="AH2" s="2" t="n"/>
+      <c r="AI2" s="2" t="n"/>
       <c r="AJ2" s="2" t="n"/>
+      <c r="AK2" s="2" t="n"/>
+      <c r="AL2" s="2" t="n"/>
+      <c r="AM2" s="3" t="n"/>
+      <c r="AN2" s="3" t="n"/>
+      <c r="AO2" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ5001"/>
+  <autoFilter ref="A1:AO5001"/>
   <dataValidations count="7">
     <dataValidation sqref="D2:D5001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$A$2:$A$4</formula1>
@@ -889,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h07 UTC</t>
+          <t>26/10/2026, 22h47 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2206,7 +2241,7 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>As colunas B, C, E, F, G, L, S, T, U e V e as ligações em W são preenchidas a partir dos dados abertos da Assembleia da República em cada captura automática. As colunas X em diante são informação adicional publicada pela AR: tema, incidência, natureza e estado da PA, avocação, identificadores e ligações. As restantes colunas do modelo (D, H a K, M a R e o texto de W) são da DACDP e nunca são alteradas pela sincronização.</t>
+          <t>As colunas B, C, E, F, G, L, S, T, U e V e as ligações em W são preenchidas a partir dos dados abertos da Assembleia da República em cada captura automática. As colunas X em diante são informação adicional publicada pela AR: tema, epígrafe, diplomas alterados, incidência, natureza e estado da PA, avocação, requerimentos, pareceres das Regiões Autónomas, identificadores e ligações. As restantes colunas do modelo (D, H a K, M a R e o texto de W) são da DACDP e nunca são alteradas pela sincronização.</t>
         </is>
       </c>
       <c r="B30" s="8" t="n"/>
@@ -3104,7 +3139,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h07 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h47 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-26 22:49 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Propostas de Alteração" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Medidas Anunciadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ponto de Situação" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Registo de Consultas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Calendário e Documentos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Resposta UPE" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas de Alteração'!$A$1:$AO$5001</definedName>
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h47 UTC</t>
+          <t>26/10/2026, 22h49 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,121 +2582,169 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E14" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3034,7 +3082,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=OsCemGn18KHljJghQ1ajbT%2fWEjfWtVhYUV7kRe%2fuHXhoN3nBlFtEOKbVu6QDIijjtsN4R56fyr1%2baHaxmvmZpOEUCWUfOUfj3wrrcEwZ7N0EVKamFEyyE1w79r%2bkbcYOysKTZQ%2frSXfq8yeBOh6uz%2bSSo7dNrYki3milkOdQK4%2fPYhVDAHRIYYyOrz9AfNYHC6%2bLY7wFcjRBgKXEr2gBz6WFsM9%2f%2bww2K4Y5MtDusKVrhlNwfEP%2bBxwqxK3ENqiwcJoPZY%2bbUiARod2nAS1emsn6ZnlYZFQfTpmOOV%2fbDqZGELEKpDw3plGCXSPbL7OVXVY4RzOCwW0D3v8CPMBJ6J1Zybv%2bENyPWZ7DPH8OTuQ%3d&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=%2fpNClpGGPpVnhbwFVXgp4qw3lFxiUpY5I8YSpeDVGH2Ez9MewVxhJZgmbME%2fa6%2bTMjV1mONPHi9qMLwrLk3vT83H5KkhIuSYQfR80BVPktegQ7Gl%2fwLhJpBRS2u1cG5OhrLVdG2YC%2bJsQxSRbcR72ynl4Szw0Kx5iDcONLD%2bGFkQ9jwIhmEnb9oj7mBISGyCnFAW%2boWpZ6JJhPzu0o0Y5y4ZJpvJ2OuBmMNL%2feYLRFY1wbMgbEZlgt35l6hrfQiWUu1j5GiKwdCYdJ9xj%2bC1ffYEAfCP0FxQup9C8cKn6PXPJ%2fcBQEZ6o%2b1Iaq9a4krvJL2CejZIuZgnT0UudK%2bZZNY47LDueTbwPwP4xVZ8KQ0J%2bQUo0RpWw0P8BT%2f3DmTE&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3056,7 +3104,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=pYwL3M4UXS4UTKShXKrBwWhp6ojHm69gObwqFN1l2E%2bxg2kG%2fhptXWmW2pG0nq46Z59GR5Hv4XPds%2bZNQrAz4A2DsnQmjHZ7PCKqj18SSwmD98VOnInmTVCdi3ITI6c4SpPPqKeXEmPQpLXOseTAjZizKS46mKyrfyKCMffvgYdbTSGC%2fbxtvJLWsGKsUDEiy0HElY9pnszJB5Bjl10iuYYp2j%2fFkyqILEqiR6F9Qx0MhMQNVRBAGgk0atcvWXLKrHuW7BV8WWt%2bQ9OGXY3m5RhVZXQ0lAc8%2bKQzNNQF1Jw271ya0A%2fQ5zo978ZcQ9MItZ6V%2fdGbJOsCxE%2filt86HDnv0Mwioj9hwHnFYJNfUgI%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=ssTiMSuZoJCViNd1vgR6NWHID3MGPk8ccDEG8T7aT7Knp0%2bD6ahQu3bm%2fXCAwHHP1m%2fLGYhARXLAI44s4yAdjFofVkflLmuhod%2fChfVb6xrtp%2fX8E1KGoSx5kEmueS0kHHfbLIBo7vFuQZD061hacolSP4UzHNsVtTsIZ%2bxqZa3NOtGWvlskniFr%2bqYioKXSCT2nZU7PsqRlrbtSWquK1%2fm5%2fSMMlkbw6t70dHBENjjqgCf6FVWAmkJfMfsWN06%2fwg1KFC9TCcBMPFlHWrC8bdy%2fMiGGFBX6YK09SuoPXLT6ExiRtSPYZpCeIB%2fZvqBhyiydH19tPstVSEMM8IKWo8Z0vwmgtxjhCAIi2zuiTBc%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -3078,7 +3126,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=Prp2%2b5ePDHjXkp5VUsQPct9bJa2RQHLO%2fyYIuha7TLAa8p6hUj1fY7Fe%2fZGk9wbXwEZmw1S14NL4ZNI8VLtcauMrxEYr0JWlnK6gPBDY3p4njYtKa%2fqnpDDAMqJEZq19UxZT6D1kt8yXuKOVU7m%2bSauySQ7xuQrqKKi11B4UGS6E%2bqkaNhmxoIqJD8U%2bCBEMrKZtj%2bAZTOvjMRpQ75atN0haT3lT67EnV7grLUcEz4%2f%2b0YUjA1h11II2KmNjheJuizQ1x3Z0c2mtgzKFJ%2fukV3duaJOIlcVz5WQbKzQvp%2fr3N7GFi3WPm15oMGmVQuTL4Iu8uiZpGwWXooc9EtWsty1Z2nzbXVJuYAv66%2f77LXc%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=fGXILUp6%2byvRm6Ifi40G9mUnq0dA55wCevtvBwtCMyx7gYlSzGO8j%2fN3obKpbXemnK2eBIpyO4lLCcO0rlA3hYaXLLW89UATI99Thh1jYaUEYYlK1%2bNIKAWZ%2fJ99%2feBnI0rhRr8020%2b4vwYeICKMx5GMs30mmbeZXKshd5E0izl2YNczd%2faDXHNQJMNQbuuXBqLXFSWZi9G2kkSltz%2bmJWmnu1W%2bRa9edq2a%2fbH1zlSEIktrSJBGGpPZVwHsz%2fOVEWMjrHQaVakyu15C1fzzMPR3BbC68LoFVnUZL%2f8xJJAWjadnHxGj7cG%2bRe42Ve4kxyzym7XK0H4drrQWGgjbZg%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3100,7 +3148,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=8VcRHu%2fGqpM4lRNrVpi9AeQ4K1Q9SnoLZ8akeOecC5sq918XRI4NEQkNDDgMmi1KupFpJ96lD21jWApIA118S9VBF4z6dlOVujEnpf2Ne3BCAIJtHbrVLchFqP%2bRWhnF%2bkAsDUaroQYYKdn0aqeiW9rRlDaUkJHWjgDNyZDu8nPITgU%2bKoG9jKrSGdrE68ioXc5QFZIbFjVs38td%2feKpMKELaoSWqIFqRqBqqyhvrXSzL%2b96AAETfgV8UkPVEmg5Wz06eSb6bsqQiuaPcs%2bOuyq9lNF1qFsUkh6H6%2bI9sJO9%2bnP%2fji0rTJramuKoYFbqHbBa6IH0aHyGMfq9JEcY8Q%3d%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=vIA7IukVsFL8hpTbQ2OM5whL1GkackwVcIcDmm6o5EWFIW5LSWyS7tEnH6b%2fJjhuVT59PCePI40rPmpxklo96oV%2bcFVfM1h7cjJ55RpcCH2VqQLpLcEaM%2fUy0Mj9%2fo12tFQ1m4960rvwIaJcQXSkd3ZraSglMqfe7kHTQr2pZhSKT%2bNuS7KluOGtL%2boO4e6PLS7%2bW8VPSJjXFJ0I3d5qUILDdrSN5BoFcS0CANXbN0d%2bbo3RoTfhTPj2ua4G3ns5RxjNRajHEgGNqtQzvpoudaIi2NIyOZD4wtCBGEpp9XkVp3wsZB9X8ge3HV7pA3eoLNEBhqAXARLQ%2btqXl5WHGJ1YmEzmS5hBbhTf2kGROOo%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3139,7 +3187,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h47 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h49 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-26 22:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h49 UTC</t>
+          <t>26/10/2026, 22h50 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -2630,121 +2630,169 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E16" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3187,7 +3235,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h49 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 22h50 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-26 23:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 22h50 UTC</t>
+          <t>26/10/2026, 23h09 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -2655,7 +2655,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -2678,121 +2678,169 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E18" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3235,7 +3283,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 22h50 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 26/10/2026, 23h09 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-27 09:37 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26/10/2026, 23h09 UTC</t>
+          <t>27/10/2026, 09h37 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -2655,7 +2655,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -2678,7 +2678,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -2726,121 +2726,169 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E20" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2865,7 +2913,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Calendário oficial e documentos publicados (situação a 26/10/2026)</t>
+          <t>Calendário oficial e documentos publicados (situação a 27/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3226,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=%2fpNClpGGPpVnhbwFVXgp4qw3lFxiUpY5I8YSpeDVGH2Ez9MewVxhJZgmbME%2fa6%2bTMjV1mONPHi9qMLwrLk3vT83H5KkhIuSYQfR80BVPktegQ7Gl%2fwLhJpBRS2u1cG5OhrLVdG2YC%2bJsQxSRbcR72ynl4Szw0Kx5iDcONLD%2bGFkQ9jwIhmEnb9oj7mBISGyCnFAW%2boWpZ6JJhPzu0o0Y5y4ZJpvJ2OuBmMNL%2feYLRFY1wbMgbEZlgt35l6hrfQiWUu1j5GiKwdCYdJ9xj%2bC1ffYEAfCP0FxQup9C8cKn6PXPJ%2fcBQEZ6o%2b1Iaq9a4krvJL2CejZIuZgnT0UudK%2bZZNY47LDueTbwPwP4xVZ8KQ0J%2bQUo0RpWw0P8BT%2f3DmTE&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=oNbIdlHa1ibAkKMS5oEWO8WVhuHdzM3zYgddvn5IuIZl7%2bCxefzuwp0JFT1a%2fJ5rFPjoJz9iji%2bMXaO15x8u4ATIFK3b54AIZlhXBVYQPGR7PU1phpF0QvTO%2bEgoNJushl6zeLvw7V%2bBPg3eHCkbtSv26WmU%2bdW%2b%2bR%2fCgUykqS9KemESBk8bNwXnMWrw53hBltqqlvv%2b18mYriwkPYWcHaAxZNVVkyljon5QvX1heu6jCX8rOCBlzQdfgIkpNN5q4OaSrwHSW5FamJPhTrmw7sz7vKRhA%2bKlUKUYvhSTCwsTBlsn2d1xCd5kNVt5T2UBqH8B1DyoPfvapERuA%2b3ReY%2bUG5TLVXT6X4Whb9lHIJCzE13P7yQTn9jikjdictNC&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3200,7 +3248,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=ssTiMSuZoJCViNd1vgR6NWHID3MGPk8ccDEG8T7aT7Knp0%2bD6ahQu3bm%2fXCAwHHP1m%2fLGYhARXLAI44s4yAdjFofVkflLmuhod%2fChfVb6xrtp%2fX8E1KGoSx5kEmueS0kHHfbLIBo7vFuQZD061hacolSP4UzHNsVtTsIZ%2bxqZa3NOtGWvlskniFr%2bqYioKXSCT2nZU7PsqRlrbtSWquK1%2fm5%2fSMMlkbw6t70dHBENjjqgCf6FVWAmkJfMfsWN06%2fwg1KFC9TCcBMPFlHWrC8bdy%2fMiGGFBX6YK09SuoPXLT6ExiRtSPYZpCeIB%2fZvqBhyiydH19tPstVSEMM8IKWo8Z0vwmgtxjhCAIi2zuiTBc%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=S7EInMa25g6onQQHeeJSi8PPPyFMm4LIFXpbpOYy0l7SMaJpvepnwt2IAVLwn575GDuwQEe2PK1hB%2fcBzV1TCeuZ4Hh2DpNoNbnk4uyf%2bTdj9OFNARWwNPV1o0HlSkQgbPAyTad849UiLQaEuPv76PLz0X8HdfkU8Dur8kvx0%2bEYyYrOKaLhVgmBBJZbpcwnEyLZ8fIZf8v9Q7h1ux4QXZvIYTHrZwaSeyJeZGHI%2buQTyf7aAwqgsoOiH7ZIjyY1DUcMHKhFNoTMiXJ69yaUVb34mJRnqCQTsNkYAkh6ggY8PVdL%2fUALKN%2bwckt%2bJUcbw6aFvXY3J0u18vD32vI%2bREl7VBpIvAJGrRiFWv3vDSurX4LICE87biJ1%2bnb2Hmk7&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -3222,7 +3270,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=fGXILUp6%2byvRm6Ifi40G9mUnq0dA55wCevtvBwtCMyx7gYlSzGO8j%2fN3obKpbXemnK2eBIpyO4lLCcO0rlA3hYaXLLW89UATI99Thh1jYaUEYYlK1%2bNIKAWZ%2fJ99%2feBnI0rhRr8020%2b4vwYeICKMx5GMs30mmbeZXKshd5E0izl2YNczd%2faDXHNQJMNQbuuXBqLXFSWZi9G2kkSltz%2bmJWmnu1W%2bRa9edq2a%2fbH1zlSEIktrSJBGGpPZVwHsz%2fOVEWMjrHQaVakyu15C1fzzMPR3BbC68LoFVnUZL%2f8xJJAWjadnHxGj7cG%2bRe42Ve4kxyzym7XK0H4drrQWGgjbZg%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=KBAUGtqy9EAWu6FgXbMPF7Zt%2f0NxOCyhLtMLZbBvVG98%2fAv2anorw49cFvrJVUyOAI5Wj9jpjwN2zeZyJWqo1%2fVBgMumo9riDk1yfzY7uLS1Ry7JZKZOzksv1PdFkJ3UCjkvYpnuL1EeGzQPnEvNIMy3FmiWCIaufnRcRfcDZxVwMlkfrvREUg76QGBm%2bTuvIeLHL8FNvpFlFwhCBoicrmUA8KzHDJnLrtbt3EP2zq43%2f34%2ftftq5vIXZBbietTAqPU1M1Kfi49erfJRXpG4hyupYvyWv8A0EiFpShkCAHQ8aq0bnf9k%2beBUJYOCEhWhwYrRxbI0FR367ji4IK3AIA%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3244,7 +3292,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=vIA7IukVsFL8hpTbQ2OM5whL1GkackwVcIcDmm6o5EWFIW5LSWyS7tEnH6b%2fJjhuVT59PCePI40rPmpxklo96oV%2bcFVfM1h7cjJ55RpcCH2VqQLpLcEaM%2fUy0Mj9%2fo12tFQ1m4960rvwIaJcQXSkd3ZraSglMqfe7kHTQr2pZhSKT%2bNuS7KluOGtL%2boO4e6PLS7%2bW8VPSJjXFJ0I3d5qUILDdrSN5BoFcS0CANXbN0d%2bbo3RoTfhTPj2ua4G3ns5RxjNRajHEgGNqtQzvpoudaIi2NIyOZD4wtCBGEpp9XkVp3wsZB9X8ge3HV7pA3eoLNEBhqAXARLQ%2btqXl5WHGJ1YmEzmS5hBbhTf2kGROOo%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=G%2fxA%2bP%2bkdXMP9dn3Xf5NMbnZ%2fWGD7e8pFoyVYH63oAochCFyqIIB8wb7HmEa2TtP%2fPEYTdhHXnFceIFz%2bPMSvs7NqGOF9qAqxnzSYtuu9MPO2q28HEL1pZDyFrITAnIHTo1xEq%2b2znOCqaaUtgxBlvTXbd1%2b9TkdxlyrThLJridqnGQscGp6TCnQjbbfsKXrFm564Oo1I%2b6XHdI4pQDwEukuwxLPqleaDqVvSA1luU%2bxMC5ub32aQLdd%2bPFuy2fnXwbrkzjFj69CRex6STn5bu0fdu6e0jFgZ%2b0nC1SbyAPoj3KYBJWCWUg1pWIJ6HSbWMZi0W6kQ%2fUNchsN2bw43A%3d%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3283,7 +3331,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 26/10/2026, 23h09 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 27/10/2026, 09h37 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-27 09:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>27/10/2026, 09h37 UTC</t>
+          <t>27/10/2026, 09h43 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:36 UTC</t>
+          <t>2026-10-27 09:42 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:36 UTC</t>
+          <t>2026-10-27 09:42 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -2655,7 +2655,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -2678,7 +2678,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -2774,121 +2774,169 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E22" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3226,7 +3274,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=oNbIdlHa1ibAkKMS5oEWO8WVhuHdzM3zYgddvn5IuIZl7%2bCxefzuwp0JFT1a%2fJ5rFPjoJz9iji%2bMXaO15x8u4ATIFK3b54AIZlhXBVYQPGR7PU1phpF0QvTO%2bEgoNJushl6zeLvw7V%2bBPg3eHCkbtSv26WmU%2bdW%2b%2bR%2fCgUykqS9KemESBk8bNwXnMWrw53hBltqqlvv%2b18mYriwkPYWcHaAxZNVVkyljon5QvX1heu6jCX8rOCBlzQdfgIkpNN5q4OaSrwHSW5FamJPhTrmw7sz7vKRhA%2bKlUKUYvhSTCwsTBlsn2d1xCd5kNVt5T2UBqH8B1DyoPfvapERuA%2b3ReY%2bUG5TLVXT6X4Whb9lHIJCzE13P7yQTn9jikjdictNC&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=dC9rQqNYGyJQXgcZhSAnCg10jPTqaC6nNvHbSBoxlSC7itNejkurPQvkBLoR%2fiIzdmTARYwM0qDkAhrWqLCSY1m8lb0PyKxiqtRMYKYVH19qcZFCCt%2fd%2frYVrmD5DVCJToMGVG8ZUuLpUYJoVVnMHhF8lySKxWp%2fzA6IXyFheQJs5qiHy7%2bXWY1LxM6B8QQRwIcKxfyNoT1B1%2fpvL3suta2wg9F4svRFG6h5369yu3p%2fBRUXlthfYX4A4Y84xqOEsmq%2bu7uBd5dflEc20bsJaLTZFDdoj6BKEfUOpWR6nrx7StxFMz1jbLbO1ja59C8m9IF6cI4vvAy%2bW6dJW7L43A4FXn29IlApHjjnnjq4lrs%3d&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3248,7 +3296,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=S7EInMa25g6onQQHeeJSi8PPPyFMm4LIFXpbpOYy0l7SMaJpvepnwt2IAVLwn575GDuwQEe2PK1hB%2fcBzV1TCeuZ4Hh2DpNoNbnk4uyf%2bTdj9OFNARWwNPV1o0HlSkQgbPAyTad849UiLQaEuPv76PLz0X8HdfkU8Dur8kvx0%2bEYyYrOKaLhVgmBBJZbpcwnEyLZ8fIZf8v9Q7h1ux4QXZvIYTHrZwaSeyJeZGHI%2buQTyf7aAwqgsoOiH7ZIjyY1DUcMHKhFNoTMiXJ69yaUVb34mJRnqCQTsNkYAkh6ggY8PVdL%2fUALKN%2bwckt%2bJUcbw6aFvXY3J0u18vD32vI%2bREl7VBpIvAJGrRiFWv3vDSurX4LICE87biJ1%2bnb2Hmk7&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=3%2fk%2bg8TKMWryONdGdPw9P9AOCwbR32Zl4rqKSmL5a7ggF1z9Z8c01T%2bzEtPFE4CVDOWR7nM5kp7%2fqpUJiMbo6xz%2bwhxPaGuYEoq2kNDlKc6JC5KVwnCRgwpm54KirCGs5MyVMLOHe82g6DzOALAIS%2bfltTcclEHevn89BXi8tbCrZGwLO11u4BoZ9w%2fccG95KsDIkw2cd%2b2wFtDxvAOBx6tP0IHv4Ilq0fgMhjDMm5jsqoAG%2bl6c6hEb1TkhAuXvx8hiapqRE8TFy53Sx9IqPyWGc6VRx7Lnra%2bvhEZJvOwpA7cxrYVEz0H%2f7Ex2TzDB1%2b6V%2bErzuLEZSOjws%2fTGrNRNu2KRpF6Iu86kaHKFmac%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -3270,7 +3318,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=KBAUGtqy9EAWu6FgXbMPF7Zt%2f0NxOCyhLtMLZbBvVG98%2fAv2anorw49cFvrJVUyOAI5Wj9jpjwN2zeZyJWqo1%2fVBgMumo9riDk1yfzY7uLS1Ry7JZKZOzksv1PdFkJ3UCjkvYpnuL1EeGzQPnEvNIMy3FmiWCIaufnRcRfcDZxVwMlkfrvREUg76QGBm%2bTuvIeLHL8FNvpFlFwhCBoicrmUA8KzHDJnLrtbt3EP2zq43%2f34%2ftftq5vIXZBbietTAqPU1M1Kfi49erfJRXpG4hyupYvyWv8A0EiFpShkCAHQ8aq0bnf9k%2beBUJYOCEhWhwYrRxbI0FR367ji4IK3AIA%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=QS08w0gPFTKQqaK0hnUDNxByJ0fgs6smsC7y90tiBLHp1ZVTB%2fwbW%2b%2fR686TNuvd%2bc%2fkPoYmTYcP1ksOX96ul%2baCRgIspms7qC2mSselXAPxdms67MGox%2bK9Yv4LrWtrk%2bm0cm3Zu0Xfqt5%2fHFYo9hPZ2XdODPZ7IeaOEdo9p%2fjV2mw56wpD2qiNbgpi6%2bd%2baKRIsBei%2fEzyasZ2wOxqXsBEnYkocDquJvv0EVAvg8irlcociBLqRoFBzi4ofxOOxnEAdWYJGWF2LJuyU7E%2bk5ZCVOONJX1AAYL7cHph86EjjGPY6Hns5DoO0wdAeoN75LeD3ixBBllODjdy3MBbAQ%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3292,7 +3340,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=G%2fxA%2bP%2bkdXMP9dn3Xf5NMbnZ%2fWGD7e8pFoyVYH63oAochCFyqIIB8wb7HmEa2TtP%2fPEYTdhHXnFceIFz%2bPMSvs7NqGOF9qAqxnzSYtuu9MPO2q28HEL1pZDyFrITAnIHTo1xEq%2b2znOCqaaUtgxBlvTXbd1%2b9TkdxlyrThLJridqnGQscGp6TCnQjbbfsKXrFm564Oo1I%2b6XHdI4pQDwEukuwxLPqleaDqVvSA1luU%2bxMC5ub32aQLdd%2bPFuy2fnXwbrkzjFj69CRex6STn5bu0fdu6e0jFgZ%2b0nC1SbyAPoj3KYBJWCWUg1pWIJ6HSbWMZi0W6kQ%2fUNchsN2bw43A%3d%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=i8w8bN%2fLuCKcExevGRu8IuUESwBkE8DS0vHHjcAoCziAx993HO0jcnymSBPeLPN5XHnDf%2bhVzBlzugGwnBqqgJ3jvOjJ5AS3bPgxeRRcQB%2fp1PzAJbyBxQqdWeojlnuPtmhL0NxJKrL6PKbV67g5TRjxnVf1iUMexlAIdgEwbFhTzSzEPYQdQ%2f625h8mZJl3UkSo81JeFKJ0tmWT7bcHGsSbV97ECES2xm6HORtkbQipDNAIc0T9cR6%2fXodDsQ4K7jzkHkQ6zk0D7x1sj4t4Hg02swr5bc15ppBA074lu%2bNMhvgSmJwwgo2TfzeqpbFGN5LwQc%2bkZOQ9GzxYNQ4seVUmcOgi%2bsOUBE5TpMAQ9v8%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3331,7 +3379,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 27/10/2026, 09h37 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 27/10/2026, 09h43 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-27 10:08 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>27/10/2026, 09h43 UTC</t>
+          <t>27/10/2026, 10h08 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:42 UTC</t>
+          <t>2026-10-27 10:07 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:42 UTC</t>
+          <t>2026-10-27 10:07 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:36 UTC</t>
+          <t>2026-10-27 09:42 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:36 UTC</t>
+          <t>2026-10-27 09:42 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -2655,7 +2655,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -2678,7 +2678,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -2774,7 +2774,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -2799,7 +2799,7 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -2822,121 +2822,169 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E24" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3379,7 +3427,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 27/10/2026, 09h43 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 27/10/2026, 10h08 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>

<commit_message>
captura 2026-10-27 10:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Registo_PA_OE2027.xlsx
+++ b/docs/Registo_PA_OE2027.xlsx
@@ -924,7 +924,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>27/10/2026, 10h08 UTC</t>
+          <t>27/10/2026, 10h50 UTC</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -2350,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 10:07 UTC</t>
+          <t>2026-10-27 10:49 UTC</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 10:07 UTC</t>
+          <t>2026-10-27 10:49 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:42 UTC</t>
+          <t>2026-10-27 10:07 UTC</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:42 UTC</t>
+          <t>2026-10-27 10:07 UTC</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:36 UTC</t>
+          <t>2026-10-27 09:42 UTC</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:36 UTC</t>
+          <t>2026-10-27 09:42 UTC</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 23:05 UTC</t>
+          <t>2026-10-27 09:36 UTC</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:49 UTC</t>
+          <t>2026-10-26 23:05 UTC</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -2655,7 +2655,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:48 UTC</t>
+          <t>2026-10-26 22:49 UTC</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -2678,7 +2678,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:06 UTC</t>
+          <t>2026-10-26 22:48 UTC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 22:00 UTC</t>
+          <t>2026-10-26 22:06 UTC</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -2774,7 +2774,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -2799,7 +2799,7 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:47 UTC</t>
+          <t>2026-10-26 22:00 UTC</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -2822,7 +2822,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -2847,7 +2847,7 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:45 UTC</t>
+          <t>2026-10-26 18:47 UTC</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -2870,121 +2870,169 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:42 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 18:41 UTC</t>
+          <t>2026-10-26 18:45 UTC</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:42 UTC</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+          <t>Portal da AR — página de cada PA (reserva)</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>0</v>
-      </c>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26 04:51 UTC</t>
+          <t>2026-10-26 18:41 UTC</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Portal da AR — página de cada PA (reserva)</t>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="n"/>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Dados abertos da AR — ficheiro de PA da edição</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/Cidadania/Paginas/DAOE.aspx</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Ficheiro da edição ainda não publicado na pasta dos dados abertos.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:51 UTC</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Portal da AR — página de cada PA (reserva)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=…</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Identificadores 25391–25415: 0 PA novas, 0 atualizadas</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
           <t>2026-10-26 04:39 UTC</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Portal da AR — pesquisa de PA</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/PesquisaPropAlteracao110XVII.aspx</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>{"disponivel": false, "erro": ""}</t>
         </is>
       </c>
-      <c r="E26" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3322,7 +3370,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=dC9rQqNYGyJQXgcZhSAnCg10jPTqaC6nNvHbSBoxlSC7itNejkurPQvkBLoR%2fiIzdmTARYwM0qDkAhrWqLCSY1m8lb0PyKxiqtRMYKYVH19qcZFCCt%2fd%2frYVrmD5DVCJToMGVG8ZUuLpUYJoVVnMHhF8lySKxWp%2fzA6IXyFheQJs5qiHy7%2bXWY1LxM6B8QQRwIcKxfyNoT1B1%2fpvL3suta2wg9F4svRFG6h5369yu3p%2fBRUXlthfYX4A4Y84xqOEsmq%2bu7uBd5dflEc20bsJaLTZFDdoj6BKEfUOpWR6nrx7StxFMz1jbLbO1ja59C8m9IF6cI4vvAy%2bW6dJW7L43A4FXn29IlApHjjnnjq4lrs%3d&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=oNbIdlHa1ibAkKMS5oEWO8WVhuHdzM3zYgddvn5IuIZl7%2bCxefzuwp0JFT1a%2fJ5rFPjoJz9iji%2bMXaO15x8u4ATIFK3b54AIZlhXBVYQPGR7PU1phpF0QvTO%2bEgoNJushl6zeLvw7V%2bBPg3eHCkbtSv26WmU%2bdW%2b%2bR%2fCgUykqS9KemESBk8bNwXnMWrw53hBltqqlvv%2b18mYriwkPYWcHaAxZNVVkyljon5QvX1heu6jCX8rOCBlzQdfgIkpNN5q4OaSrwHSW5FamJPhTrmw7sz7vKRhA%2bKlUKUYvhSTCwsTBlsn2d1xCd5kNVt5T2UBqH8B1DyoPfvapERuA%2b3ReY%2bUG5TLVXT6X4Whb9lHIJCzE13P7yQTn9jikjdictNC&amp;fich=PLOE2027_Parecer+ANMP.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3344,7 +3392,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=3%2fk%2bg8TKMWryONdGdPw9P9AOCwbR32Zl4rqKSmL5a7ggF1z9Z8c01T%2bzEtPFE4CVDOWR7nM5kp7%2fqpUJiMbo6xz%2bwhxPaGuYEoq2kNDlKc6JC5KVwnCRgwpm54KirCGs5MyVMLOHe82g6DzOALAIS%2bfltTcclEHevn89BXi8tbCrZGwLO11u4BoZ9w%2fccG95KsDIkw2cd%2b2wFtDxvAOBx6tP0IHv4Ilq0fgMhjDMm5jsqoAG%2bl6c6hEb1TkhAuXvx8hiapqRE8TFy53Sx9IqPyWGc6VRx7Lnra%2bvhEZJvOwpA7cxrYVEz0H%2f7Ex2TzDB1%2b6V%2bErzuLEZSOjws%2fTGrNRNu2KRpF6Iu86kaHKFmac%3d&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=S7EInMa25g6onQQHeeJSi8PPPyFMm4LIFXpbpOYy0l7SMaJpvepnwt2IAVLwn575GDuwQEe2PK1hB%2fcBzV1TCeuZ4Hh2DpNoNbnk4uyf%2bTdj9OFNARWwNPV1o0HlSkQgbPAyTad849UiLQaEuPv76PLz0X8HdfkU8Dur8kvx0%2bEYyYrOKaLhVgmBBJZbpcwnEyLZ8fIZf8v9Q7h1ux4QXZvIYTHrZwaSeyJeZGHI%2buQTyf7aAwqgsoOiH7ZIjyY1DUcMHKhFNoTMiXJ69yaUVb34mJRnqCQTsNkYAkh6ggY8PVdL%2fUALKN%2bwckt%2bJUcbw6aFvXY3J0u18vD32vI%2bREl7VBpIvAJGrRiFWv3vDSurX4LICE87biJ1%2bnb2Hmk7&amp;fich=CFP-REL-08-2026_POE2027.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -3366,7 +3414,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=QS08w0gPFTKQqaK0hnUDNxByJ0fgs6smsC7y90tiBLHp1ZVTB%2fwbW%2b%2fR686TNuvd%2bc%2fkPoYmTYcP1ksOX96ul%2baCRgIspms7qC2mSselXAPxdms67MGox%2bK9Yv4LrWtrk%2bm0cm3Zu0Xfqt5%2fHFYo9hPZ2XdODPZ7IeaOEdo9p%2fjV2mw56wpD2qiNbgpi6%2bd%2baKRIsBei%2fEzyasZ2wOxqXsBEnYkocDquJvv0EVAvg8irlcociBLqRoFBzi4ofxOOxnEAdWYJGWF2LJuyU7E%2bk5ZCVOONJX1AAYL7cHph86EjjGPY6Hns5DoO0wdAeoN75LeD3ixBBllODjdy3MBbAQ%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=KBAUGtqy9EAWu6FgXbMPF7Zt%2f0NxOCyhLtMLZbBvVG98%2fAv2anorw49cFvrJVUyOAI5Wj9jpjwN2zeZyJWqo1%2fVBgMumo9riDk1yfzY7uLS1Ry7JZKZOzksv1PdFkJ3UCjkvYpnuL1EeGzQPnEvNIMy3FmiWCIaufnRcRfcDZxVwMlkfrvREUg76QGBm%2bTuvIeLHL8FNvpFlFwhCBoicrmUA8KzHDJnLrtbt3EP2zq43%2f34%2ftftq5vIXZBbietTAqPU1M1Kfi49erfJRXpG4hyupYvyWv8A0EiFpShkCAHQ8aq0bnf9k%2beBUJYOCEhWhwYrRxbI0FR367ji4IK3AIA%3d%3d&amp;fich=CFP-Parecer-05-2026.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3388,7 +3436,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=i8w8bN%2fLuCKcExevGRu8IuUESwBkE8DS0vHHjcAoCziAx993HO0jcnymSBPeLPN5XHnDf%2bhVzBlzugGwnBqqgJ3jvOjJ5AS3bPgxeRRcQB%2fp1PzAJbyBxQqdWeojlnuPtmhL0NxJKrL6PKbV67g5TRjxnVf1iUMexlAIdgEwbFhTzSzEPYQdQ%2f625h8mZJl3UkSo81JeFKJ0tmWT7bcHGsSbV97ECES2xm6HORtkbQipDNAIc0T9cR6%2fXodDsQ4K7jzkHkQ6zk0D7x1sj4t4Hg02swr5bc15ppBA074lu%2bNMhvgSmJwwgo2TfzeqpbFGN5LwQc%2bkZOQ9GzxYNQ4seVUmcOgi%2bsOUBE5TpMAQ9v8%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=G%2fxA%2bP%2bkdXMP9dn3Xf5NMbnZ%2fWGD7e8pFoyVYH63oAochCFyqIIB8wb7HmEa2TtP%2fPEYTdhHXnFceIFz%2bPMSvs7NqGOF9qAqxnzSYtuu9MPO2q28HEL1pZDyFrITAnIHTo1xEq%2b2znOCqaaUtgxBlvTXbd1%2b9TkdxlyrThLJridqnGQscGp6TCnQjbbfsKXrFm564Oo1I%2b6XHdI4pQDwEukuwxLPqleaDqVvSA1luU%2bxMC5ub32aQLdd%2bPFuy2fnXwbrkzjFj69CRex6STn5bu0fdu6e0jFgZ%2b0nC1SbyAPoj3KYBJWCWUg1pWIJ6HSbWMZi0W6kQ%2fUNchsN2bw43A%3d%3d&amp;fich=Relat%c3%b3rio+UTAO.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3427,7 +3475,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 27/10/2026, 10h08 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
+          <t>Gerado automaticamente em 27/10/2026, 10h50 UTC a partir da informação publicada pela Assembleia da República. «Imediato»: preenchido em cada captura. «Desenvolvimento»: sugestão automática a validar pela DACDP. «Limitação»: sem fonte na AR.</t>
         </is>
       </c>
       <c r="B2" s="8" t="n"/>

</xml_diff>